<commit_message>
feat: Implement quiz progress tracking with Kafka integration and user progress management
</commit_message>
<xml_diff>
--- a/repo-quiz/test-data/quiz-import-chinese-full.xlsx
+++ b/repo-quiz/test-data/quiz-import-chinese-full.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DO_AN\BE_LMS\repo-quiz\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBD7770-1D08-44E3-9B37-F2FB454E37F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F78712-05C0-46DA-9E46-396A50C283B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="84">
   <si>
     <t>PackageName</t>
   </si>
@@ -28,24 +28,6 @@
     <t>PackageDescription</t>
   </si>
   <si>
-    <t>SubjectName</t>
-  </si>
-  <si>
-    <t>SubjectCode</t>
-  </si>
-  <si>
-    <t>SubjectDescription</t>
-  </si>
-  <si>
-    <t>SlotName</t>
-  </si>
-  <si>
-    <t>SlotNumber</t>
-  </si>
-  <si>
-    <t>SlotDescription</t>
-  </si>
-  <si>
     <t>FolderName</t>
   </si>
   <si>
@@ -109,22 +91,7 @@
     <t>Bo cau hoi tong hop cho ngu am, tu vung va ngu phap</t>
   </si>
   <si>
-    <t>Tieng Trung Nhap Mon</t>
-  </si>
-  <si>
-    <t>CHN101</t>
-  </si>
-  <si>
-    <t>Hoc phat am pinyin va tu vung HSK 1</t>
-  </si>
-  <si>
-    <t>Tiet 1</t>
-  </si>
-  <si>
     <t>1</t>
-  </si>
-  <si>
-    <t>On tap thanh mau va van mau</t>
   </si>
   <si>
     <t>Thu muc Tu vung va Ngu am</t>
@@ -659,37 +626,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA20"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="32" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
-    <col min="12" max="12" width="30" customWidth="1"/>
-    <col min="13" max="13" width="34" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="34" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="44" customWidth="1"/>
+    <col min="13" max="13" width="30.109375" customWidth="1"/>
+    <col min="14" max="14" width="27.21875" customWidth="1"/>
     <col min="15" max="15" width="16" customWidth="1"/>
-    <col min="16" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="18" customWidth="1"/>
-    <col min="18" max="18" width="44" customWidth="1"/>
-    <col min="19" max="19" width="30.109375" customWidth="1"/>
-    <col min="20" max="20" width="27.21875" customWidth="1"/>
-    <col min="21" max="21" width="16" customWidth="1"/>
-    <col min="22" max="22" width="26" customWidth="1"/>
-    <col min="23" max="23" width="12" customWidth="1"/>
-    <col min="24" max="25" width="16" customWidth="1"/>
-    <col min="26" max="26" width="12" customWidth="1"/>
+    <col min="16" max="16" width="26" customWidth="1"/>
+    <col min="17" max="17" width="12" customWidth="1"/>
+    <col min="18" max="19" width="16" customWidth="1"/>
+    <col min="20" max="20" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -753,331 +714,295 @@
       <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="B2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q3" t="s">
+        <v>39</v>
+      </c>
+      <c r="R3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q4" t="s">
+        <v>41</v>
+      </c>
+      <c r="R4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q5" t="s">
+        <v>42</v>
+      </c>
+      <c r="R5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="L6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O6" t="s">
+        <v>36</v>
+      </c>
+      <c r="P6" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>45</v>
+      </c>
+      <c r="R6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q7" t="s">
+        <v>46</v>
+      </c>
+      <c r="R7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q8" t="s">
+        <v>47</v>
+      </c>
+      <c r="R8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q9" t="s">
+        <v>48</v>
+      </c>
+      <c r="R9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="L10" t="s">
+        <v>49</v>
+      </c>
+      <c r="M10" t="s">
+        <v>50</v>
+      </c>
+      <c r="N10" t="s">
+        <v>51</v>
+      </c>
+      <c r="O10" t="s">
+        <v>36</v>
+      </c>
+      <c r="P10" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>53</v>
+      </c>
+      <c r="R10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q11" t="s">
+        <v>55</v>
+      </c>
+      <c r="R11" t="s">
+        <v>56</v>
+      </c>
+      <c r="S11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="L12" t="s">
+        <v>58</v>
+      </c>
+      <c r="M12" t="s">
+        <v>59</v>
+      </c>
+      <c r="N12" t="s">
+        <v>60</v>
+      </c>
+      <c r="O12" t="s">
+        <v>36</v>
+      </c>
+      <c r="P12" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>61</v>
+      </c>
+      <c r="R12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q13" t="s">
+        <v>63</v>
+      </c>
+      <c r="R13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="M14" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>65</v>
+      </c>
+      <c r="R14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Q15" t="s">
+        <v>67</v>
+      </c>
+      <c r="R15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="L16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M16" t="s">
+        <v>70</v>
+      </c>
+      <c r="N16" t="s">
+        <v>71</v>
+      </c>
+      <c r="O16" t="s">
+        <v>36</v>
+      </c>
+      <c r="P16" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>73</v>
+      </c>
+      <c r="R16" t="s">
+        <v>74</v>
+      </c>
+      <c r="S16" t="s">
+        <v>75</v>
+      </c>
+      <c r="T16" t="s">
+        <v>76</v>
+      </c>
+      <c r="U16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="Q17" t="s">
+        <v>77</v>
+      </c>
+      <c r="S17" t="s">
+        <v>55</v>
+      </c>
+      <c r="T17" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" t="s">
-        <v>35</v>
-      </c>
-      <c r="J2" t="s">
-        <v>36</v>
-      </c>
-      <c r="K2" t="s">
-        <v>37</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="U17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="S18" t="s">
+        <v>78</v>
+      </c>
+      <c r="T18" t="s">
+        <v>79</v>
+      </c>
+      <c r="U18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="S19" t="s">
+        <v>80</v>
+      </c>
+      <c r="T19" t="s">
+        <v>81</v>
+      </c>
+      <c r="U19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="S20" t="s">
+        <v>82</v>
+      </c>
+      <c r="T20" t="s">
+        <v>83</v>
+      </c>
+      <c r="U20" t="s">
         <v>38</v>
-      </c>
-      <c r="M2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N2" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" t="s">
-        <v>41</v>
-      </c>
-      <c r="P2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>43</v>
-      </c>
-      <c r="R2" t="s">
-        <v>44</v>
-      </c>
-      <c r="S2" t="s">
-        <v>45</v>
-      </c>
-      <c r="T2" t="s">
-        <v>46</v>
-      </c>
-      <c r="U2" t="s">
-        <v>47</v>
-      </c>
-      <c r="V2" t="s">
-        <v>41</v>
-      </c>
-      <c r="W2" t="s">
-        <v>48</v>
-      </c>
-      <c r="X2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W3" t="s">
-        <v>50</v>
-      </c>
-      <c r="X3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W4" t="s">
-        <v>52</v>
-      </c>
-      <c r="X4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W5" t="s">
-        <v>53</v>
-      </c>
-      <c r="X5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="R6" t="s">
-        <v>44</v>
-      </c>
-      <c r="S6" t="s">
-        <v>54</v>
-      </c>
-      <c r="T6" t="s">
-        <v>55</v>
-      </c>
-      <c r="U6" t="s">
-        <v>47</v>
-      </c>
-      <c r="V6" t="s">
-        <v>41</v>
-      </c>
-      <c r="W6" t="s">
-        <v>56</v>
-      </c>
-      <c r="X6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W7" t="s">
-        <v>57</v>
-      </c>
-      <c r="X7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W8" t="s">
-        <v>58</v>
-      </c>
-      <c r="X8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W9" t="s">
-        <v>59</v>
-      </c>
-      <c r="X9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="R10" t="s">
-        <v>60</v>
-      </c>
-      <c r="S10" t="s">
-        <v>61</v>
-      </c>
-      <c r="T10" t="s">
-        <v>62</v>
-      </c>
-      <c r="U10" t="s">
-        <v>47</v>
-      </c>
-      <c r="V10" t="s">
-        <v>63</v>
-      </c>
-      <c r="W10" t="s">
-        <v>64</v>
-      </c>
-      <c r="X10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W11" t="s">
-        <v>66</v>
-      </c>
-      <c r="X11" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y11" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="R12" t="s">
-        <v>69</v>
-      </c>
-      <c r="S12" t="s">
-        <v>70</v>
-      </c>
-      <c r="T12" t="s">
-        <v>71</v>
-      </c>
-      <c r="U12" t="s">
-        <v>47</v>
-      </c>
-      <c r="V12" t="s">
-        <v>63</v>
-      </c>
-      <c r="W12" t="s">
-        <v>72</v>
-      </c>
-      <c r="X12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W13" t="s">
-        <v>74</v>
-      </c>
-      <c r="X13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="S14" t="s">
-        <v>70</v>
-      </c>
-      <c r="W14" t="s">
-        <v>76</v>
-      </c>
-      <c r="X14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W15" t="s">
-        <v>78</v>
-      </c>
-      <c r="X15" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="R16" t="s">
-        <v>80</v>
-      </c>
-      <c r="S16" t="s">
-        <v>81</v>
-      </c>
-      <c r="T16" t="s">
-        <v>82</v>
-      </c>
-      <c r="U16" t="s">
-        <v>47</v>
-      </c>
-      <c r="V16" t="s">
-        <v>83</v>
-      </c>
-      <c r="W16" t="s">
-        <v>84</v>
-      </c>
-      <c r="X16" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y16" t="s">
-        <v>86</v>
-      </c>
-      <c r="Z16" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="W17" t="s">
-        <v>88</v>
-      </c>
-      <c r="Y17" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z17" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA17" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="Y18" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z18" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA18" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="Y19" t="s">
-        <v>91</v>
-      </c>
-      <c r="Z19" t="s">
-        <v>92</v>
-      </c>
-      <c r="AA19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="20" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="Y20" t="s">
-        <v>93</v>
-      </c>
-      <c r="Z20" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA20" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>